<commit_message>
Post-audit revision: sanitizer-confirm F-07, report filtered coverage, fix overclaims
- Run SQE-PRB-05/06 under ASan/UBSan (tools/sqe_asan_probes.sh, tools/sqe_ubsan_probes.sh):
  F-07a ASan stack-buffer-overflow at FailureInjector.cpp:118, F-07b UBSan shift exponent at :120.
  Workbook now reports these probes as FAIL with sanitizer evidence instead of an inert PASS.
- Report exception-filtered branch coverage (376/384, 97.9%) next to the raw 82.3%;
  fix GAPS.md's claim that feasible numbers already existed.
- MC/DC wording: "unique-cause under short-circuit relaxation", not "no masking throughout".
- F-09/F-10 relabelled candidate defects pending team review.
- SQE-DVG-12: replace bare SUCCEED() with real oracles; coverage unchanged; patch regenerated.
- .gitattributes: keep *.patch LF so it applies on Windows clones.
- Add independent second-machine reproduction evidence (identical coverage hit sets).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/24i3015_24i3166_24i3158_B.xlsx
+++ b/deliverables/24i3015_24i3166_24i3158_B.xlsx
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>expected conf&lt;1 under a stricter spec; contradicts confirmed F-09 characterization (conf=1) -- oracle approved as the correct reading 2026-10-01 (F-09 resolved as a confirmed defect)</t>
+          <t>expected conf&lt;1 under a stricter spec; contradicts confirmed F-09 characterization (conf=1) -- stricter oracle proposed 2026-10-01 (F-09 candidate defect, pending whole-team review)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>expected state!=0 under a stricter spec; contradicts confirmed F-10 characterization (state=0) -- oracle approved as the correct reading 2026-10-01 (F-10 resolved as a confirmed defect)</t>
+          <t>expected state!=0 under a stricter spec; contradicts confirmed F-10 characterization (state=0) -- stricter oracle proposed 2026-10-01 (F-10 candidate defect, pending whole-team review)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Construct/destroy groups of size 0..5 (one with an extra add_new_validator()) without crashing</t>
+          <t>Constructor links exactly n siblings for sizes 0..5; add_new_validator() appends a reachable sibling; destructor walks every sibling (smoke)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>no crash</t>
+          <t>get_sensor_state(i)!=UINT32_MAX for all i&lt;n and ==UINT32_MAX at i==n; after add_new_validator() on g(3): index 3 found, index 4 not found; destructor runs without crash (freeing not observable via API) [DataValidatorGroup.cpp L54-65, L74-80, L83-95, L313-328]</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>DVG-D04</t>
+          <t>DVG-D01 T/F; DVG-D02 T/F; DVG-D04; DVG-D35/D36 T/F</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -5313,12 +5313,12 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>expected: ASan-detected out-of-bounds write on esc[8] (only observable under ASan, confirmed real defect per work/basis/INVENTORY)</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>under ASan: the probe aborts with stack-buffer-overflow, READ at FailureInjector.cpp:118 (status.esc[8], one past the esc[8] array) -&gt; F-07a defect present. In a normal/Coverage build the probe is an inert SUCCEED() and proves nothing</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>FailureInjector.cpp ; evidence/tests/probes/functional-SqeFailureInjector_PRB0506.xml</t>
+          <t>FailureInjector.cpp ; sanitizer run: evidence/tests/sanitizer/asan_PRB05.log (ASan stack-buffer-overflow at FailureInjector.cpp:118; reproduce with tools/sqe_asan_probes.sh) -- fails as expected, defect F-07a confirmed at runtime</t>
         </is>
       </c>
     </row>
@@ -5355,12 +5355,12 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>expected: UBSan-detected 'shift exponent too large' (only observable under UBSan, confirmed real defect per work/basis/INVENTORY)</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>under UBSan (-fsanitize=shift): 'shift exponent 4294967195 is too large for 32-bit type int' at FailureInjector.cpp:120 -&gt; F-07b defect present. In a normal/Coverage build the probe is an inert SUCCEED() and proves nothing</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>FailureInjector.cpp ; evidence/tests/probes/functional-SqeFailureInjector_PRB0506.xml</t>
+          <t>FailureInjector.cpp ; sanitizer run: evidence/tests/sanitizer/ubsan_PRB06.log (UBSan shift-exponent runtime error at FailureInjector.cpp:120; reproduce with tools/sqe_ubsan_probes.sh) -- fails as expected, defect F-07b confirmed at runtime</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
@@ -6202,7 +6202,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
@@ -6299,7 +6299,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
@@ -7416,7 +7416,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr">
@@ -8145,7 +8145,7 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>unique-cause</t>
+          <t>unique-cause (short-circuit)</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">

</xml_diff>